<commit_message>
Updated sourcing page UI
</commit_message>
<xml_diff>
--- a/wishlist.xlsx
+++ b/wishlist.xlsx
@@ -501,10 +501,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>RS Components</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -543,17 +547,25 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>resistor</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+          <t>RESISTOR</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>BHJ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>10k</t>
+        </is>
+      </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -569,29 +581,21 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RESISTOR</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>BHJ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>10k</t>
-        </is>
-      </c>
+          <t>lm358</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -612,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -693,6 +697,41 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>RS Components</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Trusted</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>